<commit_message>
Add DAM image package for design pages; keep Tata Cars logos through Content Sync
- tools/aem-packages: CRX content package with the 65 design images (DAM folder exp-mord-agent) and a plain-folder zip, plus the build script
- header: an unlinked logo next to the brand link becomes the link content (linked images are dropped by Content Sync)
- Tata Cars nav/footer re-imported with unlinked logos

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-tatacars.report.xlsx
+++ b/tools/importer/reports/import-tatacars.report.xlsx
@@ -229,7 +229,7 @@
     <t>tata-cars-footer</t>
   </si>
   <si>
-    <t>2026-10-08T06:33:05.150Z</t>
+    <t>2026-10-08T07:11:36.308Z</t>
   </si>
   <si>
     <t>Tata Cars footer fragment: brand, newsletter (form-contact), range + links, contact + social</t>
@@ -244,7 +244,7 @@
     <t>tata-cars-nav</t>
   </si>
   <si>
-    <t>2026-10-08T06:33:00.408Z</t>
+    <t>2026-10-08T07:11:31.607Z</t>
   </si>
   <si>
     <t>Tata Cars header fragment: brand | sections | tools</t>
@@ -262,7 +262,7 @@
     <t>tata-cars</t>
   </si>
   <si>
-    <t>2026-10-08T06:32:53.985Z</t>
+    <t>2026-10-08T07:11:27.693Z</t>
   </si>
   <si>
     <t>TATA.CARS | Skip the waitlist. Secure yours today.</t>

</xml_diff>